<commit_message>
fix: rename Bangles to Bracelet globally in categories and products databases and update backend synonyms
</commit_message>
<xml_diff>
--- a/server/database/products.xlsx
+++ b/server/database/products.xlsx
@@ -486,7 +486,7 @@
         <v>47300</v>
       </c>
       <c r="F3" t="str">
-        <v>Bangles</v>
+        <v>Bracelet</v>
       </c>
       <c r="G3" t="str">
         <v>["https://images.unsplash.com/photo-1611591437281-460bfbe1220a?w=600&amp;auto=format&amp;fit=crop&amp;q=80","https://images.unsplash.com/photo-1535632066927-ab7c9ab60908?w=600&amp;auto=format&amp;fit=crop&amp;q=80"]</v>
@@ -626,7 +626,7 @@
         <v>42914</v>
       </c>
       <c r="F7" t="str">
-        <v>Bangles</v>
+        <v>Bracelet</v>
       </c>
       <c r="G7" t="str">
         <v>["https://images.unsplash.com/photo-1535632066927-ab7c9ab60908?w=600&amp;auto=format&amp;fit=crop&amp;q=80"]</v>

</xml_diff>